<commit_message>
fix: AchieveManager 버그 수정. refactor: Singleton.Awake() 구조 변경.
</commit_message>
<xml_diff>
--- a/input/Domains/Game/GameTable.xlsx
+++ b/input/Domains/Game/GameTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maoshy/Documents/Projects/devian/input/Domains/Game/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E616A610-9987-1E4A-908E-076745AB5CCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E753E76-16A3-904D-B7CE-445AEB313F2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1380" yWindow="500" windowWidth="37020" windowHeight="21100" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1380" yWindow="500" windowWidth="37020" windowHeight="21100" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MESSAGE" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="119">
   <si>
     <t>messageId</t>
   </si>
@@ -224,6 +224,9 @@
     <t>achieveId</t>
   </si>
   <si>
+    <t>achieveType</t>
+  </si>
+  <si>
     <t>level</t>
   </si>
   <si>
@@ -233,17 +236,23 @@
     <t>googleAchievementId</t>
   </si>
   <si>
+    <t>ACHIEVE_TYPE</t>
+  </si>
+  <si>
     <t>group:true</t>
   </si>
   <si>
     <t>내부 업적 ID (정본)</t>
   </si>
   <si>
+    <t>업적 타입 (DEFAULT=자동 런타임 생성)</t>
+  </si>
+  <si>
     <t>업적 단계</t>
   </si>
   <si>
     <t>UI 정렬 기준 값 (1부터 시작)._x000D__x000D_
-같은 missionId group은 같은 값을 사용한다.</t>
+같은 achieveId group은 같은 값을 사용한다.</t>
   </si>
   <si>
     <t>MESSAGE.messageId (정본, source: MESSAGE)</t>
@@ -253,16 +262,16 @@
 {base, pow}</t>
   </si>
   <si>
-    <t>Apple Game Center Achievement ID (missionId group 공통)</t>
-  </si>
-  <si>
-    <t>Google Play Games Achievement ID (missionId group 공통)</t>
+    <t>Apple Game Center Achievement ID (achieveId group 공통)</t>
+  </si>
+  <si>
+    <t>Google Play Games Achievement ID (achieveId group 공통)</t>
   </si>
   <si>
     <t>achieve_001</t>
   </si>
   <si>
-    <t>{100, 0}</t>
+    <t>DEFAULT</t>
   </si>
   <si>
     <t>reward_mission_achieve_001</t>
@@ -271,27 +280,15 @@
     <t>CgkIi_C0k7wDEAIQBg</t>
   </si>
   <si>
-    <t>{300, 0}</t>
-  </si>
-  <si>
     <t>reward_mission_achieve_002</t>
   </si>
   <si>
-    <t>{1000, 0}</t>
-  </si>
-  <si>
     <t>reward_mission_achieve_003</t>
   </si>
   <si>
-    <t>{5000, 0}</t>
-  </si>
-  <si>
     <t>reward_mission_achieve_004</t>
   </si>
   <si>
-    <t>{30000, 0}</t>
-  </si>
-  <si>
     <t>reward_mission_achieve_005</t>
   </si>
   <si>
@@ -386,10 +383,6 @@
   </si>
   <si>
     <t>inclusive end rank</t>
-  </si>
-  <si>
-    <t>reward_mission_achieve_004</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1177,7 +1170,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
   <cols>
     <col min="2" max="2" width="18.28515625" bestFit="1" customWidth="1"/>
@@ -1188,7 +1181,7 @@
     <col min="10" max="10" width="27.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:11">
       <c r="A1" t="s">
         <v>64</v>
       </c>
@@ -1196,31 +1189,34 @@
         <v>65</v>
       </c>
       <c r="C1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D1" t="s">
         <v>37</v>
       </c>
-      <c r="D1" t="s">
-        <v>66</v>
-      </c>
       <c r="E1" t="s">
+        <v>67</v>
+      </c>
+      <c r="F1" t="s">
         <v>39</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>0</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>40</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>41</v>
-      </c>
-      <c r="I1" t="s">
-        <v>67</v>
       </c>
       <c r="J1" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="2" spans="1:10">
+      <c r="K1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
       <c r="A2" t="s">
         <v>44</v>
       </c>
@@ -1228,302 +1224,335 @@
         <v>3</v>
       </c>
       <c r="C2" t="s">
+        <v>70</v>
+      </c>
+      <c r="D2" t="s">
         <v>43</v>
-      </c>
-      <c r="D2" t="s">
-        <v>44</v>
       </c>
       <c r="E2" t="s">
         <v>44</v>
       </c>
       <c r="F2" t="s">
-        <v>3</v>
+        <v>44</v>
       </c>
       <c r="G2" t="s">
+        <v>3</v>
+      </c>
+      <c r="H2" t="s">
         <v>45</v>
       </c>
-      <c r="H2" t="s">
-        <v>3</v>
-      </c>
       <c r="I2" t="s">
         <v>3</v>
       </c>
       <c r="J2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:10">
+      <c r="K2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
       <c r="A3" t="s">
         <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
       <c r="B4" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C4" t="s">
+        <v>73</v>
+      </c>
+      <c r="D4" t="s">
         <v>47</v>
       </c>
-      <c r="D4" t="s">
-        <v>71</v>
-      </c>
       <c r="E4" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F4" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="G4" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H4" t="s">
+        <v>77</v>
+      </c>
+      <c r="I4" t="s">
         <v>52</v>
       </c>
-      <c r="I4" t="s">
-        <v>75</v>
-      </c>
       <c r="J4" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10">
+        <v>78</v>
+      </c>
+      <c r="K4" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
       <c r="A5">
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>77</v>
-      </c>
-      <c r="C5" t="b">
-        <v>1</v>
-      </c>
-      <c r="D5">
+        <v>80</v>
+      </c>
+      <c r="C5" t="s">
+        <v>81</v>
+      </c>
+      <c r="D5" t="b">
         <v>1</v>
       </c>
       <c r="E5">
         <v>1</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5" t="s">
         <v>10</v>
       </c>
-      <c r="G5" t="s">
-        <v>78</v>
-      </c>
-      <c r="H5" t="s">
-        <v>79</v>
-      </c>
-      <c r="J5" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10">
+      <c r="H5">
+        <v>10</v>
+      </c>
+      <c r="I5" t="s">
+        <v>82</v>
+      </c>
+      <c r="K5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
       <c r="A6">
         <v>2</v>
       </c>
       <c r="B6" t="s">
-        <v>77</v>
-      </c>
-      <c r="C6" t="b">
-        <v>1</v>
-      </c>
-      <c r="D6">
+        <v>80</v>
+      </c>
+      <c r="C6" t="s">
+        <v>81</v>
+      </c>
+      <c r="D6" t="b">
+        <v>1</v>
+      </c>
+      <c r="E6">
         <v>2</v>
       </c>
-      <c r="E6">
-        <v>1</v>
-      </c>
-      <c r="F6" t="s">
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6" t="s">
         <v>10</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6">
+        <v>40</v>
+      </c>
+      <c r="I6" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
+      <c r="A7">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>80</v>
+      </c>
+      <c r="C7" t="s">
         <v>81</v>
       </c>
-      <c r="H6" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10">
-      <c r="A7">
-        <v>3</v>
-      </c>
-      <c r="B7" t="s">
-        <v>77</v>
-      </c>
-      <c r="C7" t="b">
-        <v>1</v>
-      </c>
-      <c r="D7">
-        <v>3</v>
+      <c r="D7" t="b">
+        <v>1</v>
       </c>
       <c r="E7">
-        <v>1</v>
-      </c>
-      <c r="F7" t="s">
+        <v>3</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7" t="s">
         <v>10</v>
       </c>
-      <c r="G7" t="s">
-        <v>83</v>
-      </c>
-      <c r="H7" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10">
+      <c r="H7">
+        <v>200</v>
+      </c>
+      <c r="I7" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
       <c r="A8">
         <v>4</v>
       </c>
       <c r="B8" t="s">
-        <v>77</v>
-      </c>
-      <c r="C8" t="b">
-        <v>1</v>
-      </c>
-      <c r="D8">
+        <v>80</v>
+      </c>
+      <c r="C8" t="s">
+        <v>81</v>
+      </c>
+      <c r="D8" t="b">
+        <v>1</v>
+      </c>
+      <c r="E8">
         <v>4</v>
       </c>
-      <c r="E8">
-        <v>1</v>
-      </c>
-      <c r="F8" t="s">
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8" t="s">
         <v>10</v>
       </c>
-      <c r="G8" t="s">
-        <v>85</v>
-      </c>
-      <c r="H8" t="s">
+      <c r="H8">
+        <v>1000</v>
+      </c>
+      <c r="I8" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:11">
       <c r="A9">
         <v>5</v>
       </c>
       <c r="B9" t="s">
-        <v>77</v>
-      </c>
-      <c r="C9" t="b">
-        <v>1</v>
-      </c>
-      <c r="D9">
+        <v>80</v>
+      </c>
+      <c r="C9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D9" t="b">
+        <v>1</v>
+      </c>
+      <c r="E9">
         <v>5</v>
       </c>
-      <c r="E9">
-        <v>1</v>
-      </c>
-      <c r="F9" t="s">
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9" t="s">
         <v>10</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9">
+        <v>5000</v>
+      </c>
+      <c r="I9" t="s">
         <v>87</v>
       </c>
-      <c r="H9" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10">
+    </row>
+    <row r="10" spans="1:11">
       <c r="A10">
         <v>6</v>
       </c>
       <c r="B10" t="s">
-        <v>89</v>
-      </c>
-      <c r="C10" t="b">
-        <v>1</v>
-      </c>
-      <c r="D10">
+        <v>88</v>
+      </c>
+      <c r="C10" t="s">
+        <v>81</v>
+      </c>
+      <c r="D10" t="b">
         <v>1</v>
       </c>
       <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="F10">
         <v>2</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>13</v>
       </c>
-      <c r="G10">
+      <c r="H10">
         <v>100</v>
       </c>
-      <c r="H10" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10">
+      <c r="I10" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11">
       <c r="A11">
         <v>7</v>
       </c>
       <c r="B11" t="s">
-        <v>90</v>
-      </c>
-      <c r="C11" t="b">
-        <v>1</v>
-      </c>
-      <c r="D11">
+        <v>89</v>
+      </c>
+      <c r="C11" t="s">
+        <v>81</v>
+      </c>
+      <c r="D11" t="b">
         <v>1</v>
       </c>
       <c r="E11">
-        <v>3</v>
-      </c>
-      <c r="F11" t="s">
+        <v>1</v>
+      </c>
+      <c r="F11">
+        <v>3</v>
+      </c>
+      <c r="G11" t="s">
         <v>15</v>
       </c>
-      <c r="G11">
+      <c r="H11">
         <v>100</v>
       </c>
-      <c r="H11" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10">
+      <c r="I11" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11">
       <c r="A12">
         <v>8</v>
       </c>
       <c r="B12" t="s">
-        <v>91</v>
-      </c>
-      <c r="C12" t="b">
-        <v>1</v>
-      </c>
-      <c r="D12">
+        <v>90</v>
+      </c>
+      <c r="C12" t="s">
+        <v>81</v>
+      </c>
+      <c r="D12" t="b">
         <v>1</v>
       </c>
       <c r="E12">
+        <v>1</v>
+      </c>
+      <c r="F12">
         <v>4</v>
       </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
         <v>17</v>
       </c>
-      <c r="G12">
+      <c r="H12">
         <v>100</v>
       </c>
-      <c r="H12" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10">
+      <c r="I12" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11">
       <c r="A13">
         <v>9</v>
       </c>
       <c r="B13" t="s">
-        <v>92</v>
-      </c>
-      <c r="C13" t="b">
-        <v>1</v>
-      </c>
-      <c r="D13">
+        <v>91</v>
+      </c>
+      <c r="C13" t="s">
+        <v>81</v>
+      </c>
+      <c r="D13" t="b">
         <v>1</v>
       </c>
       <c r="E13">
+        <v>1</v>
+      </c>
+      <c r="F13">
         <v>5</v>
       </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
         <v>19</v>
       </c>
-      <c r="G13">
+      <c r="H13">
         <v>100</v>
       </c>
-      <c r="H13" t="s">
-        <v>88</v>
+      <c r="I13" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>
@@ -1547,7 +1576,7 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B1" t="s">
         <v>37</v>
@@ -1556,22 +1585,22 @@
         <v>0</v>
       </c>
       <c r="D1" t="s">
+        <v>93</v>
+      </c>
+      <c r="E1" t="s">
         <v>94</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>95</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>96</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>97</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>98</v>
-      </c>
-      <c r="I1" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -1594,13 +1623,13 @@
         <v>3</v>
       </c>
       <c r="G2" t="s">
+        <v>99</v>
+      </c>
+      <c r="H2" t="s">
         <v>100</v>
       </c>
-      <c r="H2" t="s">
-        <v>101</v>
-      </c>
       <c r="I2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -1610,36 +1639,36 @@
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B4" t="s">
         <v>47</v>
       </c>
       <c r="C4" t="s">
+        <v>102</v>
+      </c>
+      <c r="D4" t="s">
         <v>103</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>104</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>105</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>106</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>107</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>108</v>
-      </c>
-      <c r="I4" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="19" customHeight="1">
       <c r="A5" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B5" t="b">
         <v>1</v>
@@ -1648,13 +1677,13 @@
         <v>32</v>
       </c>
       <c r="E5" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="F5" t="s">
         <v>111</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>112</v>
-      </c>
-      <c r="G5" t="s">
-        <v>113</v>
       </c>
       <c r="H5">
         <v>1767225600000</v>
@@ -1683,13 +1712,13 @@
         <v>64</v>
       </c>
       <c r="B1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C1" t="s">
+        <v>113</v>
+      </c>
+      <c r="D1" t="s">
         <v>114</v>
-      </c>
-      <c r="D1" t="s">
-        <v>115</v>
       </c>
       <c r="E1" t="s">
         <v>41</v>
@@ -1703,10 +1732,10 @@
         <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E2" t="s">
         <v>3</v>
@@ -1717,21 +1746,21 @@
         <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
+        <v>115</v>
+      </c>
+      <c r="B4" t="s">
         <v>116</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>117</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>118</v>
-      </c>
-      <c r="D4" t="s">
-        <v>119</v>
       </c>
       <c r="E4" t="s">
         <v>52</v>
@@ -1742,7 +1771,7 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C5">
         <v>1</v>
@@ -1751,7 +1780,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="s">
-        <v>120</v>
+        <v>86</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -1759,7 +1788,7 @@
         <v>2</v>
       </c>
       <c r="B6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C6">
         <v>11</v>
@@ -1768,7 +1797,7 @@
         <v>100</v>
       </c>
       <c r="E6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feature: Achieve에 시작 조건 추가.
</commit_message>
<xml_diff>
--- a/input/Domains/Game/GameTable.xlsx
+++ b/input/Domains/Game/GameTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maoshy/Documents/Projects/devian/input/Domains/Game/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{116CEA10-0F13-0A4E-BB06-43C4E45AF3FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8C70C25-2465-FF47-AF88-CED85B51CD56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1380" yWindow="500" windowWidth="37020" windowHeight="21100" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1320" yWindow="500" windowWidth="37080" windowHeight="21100" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MESSAGE" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="133">
   <si>
     <t>messageId</t>
   </si>
@@ -131,6 +131,36 @@
     <t>TOTAL_MAX</t>
   </si>
   <si>
+    <t>msg_battle_pass_001</t>
+  </si>
+  <si>
+    <t>BATTLE_PASS_001</t>
+  </si>
+  <si>
+    <t>msg_battle_pass_002</t>
+  </si>
+  <si>
+    <t>BATTLE_PASS_002</t>
+  </si>
+  <si>
+    <t>msg_battle_pass_003</t>
+  </si>
+  <si>
+    <t>BATTLE_PASS_003</t>
+  </si>
+  <si>
+    <t>msg_battle_pass_004</t>
+  </si>
+  <si>
+    <t>BATTLE_PASS_004</t>
+  </si>
+  <si>
+    <t>msg_battle_pass_005</t>
+  </si>
+  <si>
+    <t>BATTLE_PASS_005</t>
+  </si>
+  <si>
     <t>missionId</t>
   </si>
   <si>
@@ -230,6 +260,15 @@
     <t>level</t>
   </si>
   <si>
+    <t>reqMsgId</t>
+  </si>
+  <si>
+    <t>reqValue</t>
+  </si>
+  <si>
+    <t>conditionMsgId</t>
+  </si>
+  <si>
     <t>appleAchievementId</t>
   </si>
   <si>
@@ -242,6 +281,9 @@
     <t>group:true</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>내부 업적 ID (정본)</t>
   </si>
   <si>
@@ -251,14 +293,11 @@
     <t>업적 단계</t>
   </si>
   <si>
-    <t>UI 정렬 기준 값 (1부터 시작)._x000D__x000D__x000D_
+    <t>UI 정렬 기준 값 (1부터 시작)._x000D__x000D__x000D__x000D__x000D_
 같은 achieveId group은 같은 값을 사용한다.</t>
   </si>
   <si>
-    <t>MESSAGE.messageId (정본, source: MESSAGE)</t>
-  </si>
-  <si>
-    <t>조건 목표값_x000D__x000D_
+    <t>조건 목표값_x000D__x000D__x000D__x000D_
 {base, pow}</t>
   </si>
   <si>
@@ -274,6 +313,9 @@
     <t>DEFAULT</t>
   </si>
   <si>
+    <t>1</t>
+  </si>
+  <si>
     <t>reward_mission_achieve_001</t>
   </si>
   <si>
@@ -307,24 +349,21 @@
     <t>leaderboardId</t>
   </si>
   <si>
+    <t>mode</t>
+  </si>
+  <si>
+    <t>seasonStartUtc</t>
+  </si>
+  <si>
+    <t>seasonEndUtc</t>
+  </si>
+  <si>
     <t>appleLeaderboardId</t>
   </si>
   <si>
     <t>googleLeaderboardId</t>
   </si>
   <si>
-    <t>seasonId</t>
-  </si>
-  <si>
-    <t>mode</t>
-  </si>
-  <si>
-    <t>seasonStartUtc</t>
-  </si>
-  <si>
-    <t>seasonEndUtc</t>
-  </si>
-  <si>
     <t>LEADERBOARD_MODE</t>
   </si>
   <si>
@@ -337,40 +376,34 @@
     <t>MESSAGE.messageId (score source)</t>
   </si>
   <si>
+    <t>리더보드 모드</t>
+  </si>
+  <si>
+    <t>시즌 시작 UTC ms</t>
+  </si>
+  <si>
+    <t>시즌 종료 UTC ms</t>
+  </si>
+  <si>
     <t>Apple Game Center Leaderboard ID</t>
   </si>
   <si>
     <t>Google Play Games Leaderboard ID</t>
   </si>
   <si>
-    <t>시즌 식별자</t>
-  </si>
-  <si>
-    <t>리더보드 모드</t>
-  </si>
-  <si>
-    <t>시즌 시작 UTC ms</t>
-  </si>
-  <si>
-    <t>시즌 종료 UTC ms</t>
-  </si>
-  <si>
     <t>leaderboard_001</t>
   </si>
   <si>
+    <t>NORMAL</t>
+  </si>
+  <si>
+    <t>2026-01-01 00:00:00.000</t>
+  </si>
+  <si>
+    <t>2026-04-01 00:00:00.000</t>
+  </si>
+  <si>
     <t>CgkIi_C0k7wDEAIQBw</t>
-  </si>
-  <si>
-    <t>s2026_q1</t>
-  </si>
-  <si>
-    <t>NORMAL</t>
-  </si>
-  <si>
-    <t>2026-01-01 00:00:00.000</t>
-  </si>
-  <si>
-    <t>2026-04-01 00:00:00.000</t>
   </si>
   <si>
     <t>rankFrom</t>
@@ -775,7 +808,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -937,11 +970,66 @@
         <v>34</v>
       </c>
     </row>
+    <row r="16" spans="1:3">
+      <c r="A16" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B17" t="s">
+        <v>38</v>
+      </c>
+      <c r="C17" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" t="s">
+        <v>39</v>
+      </c>
+      <c r="B18" t="s">
+        <v>40</v>
+      </c>
+      <c r="C18" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" t="s">
+        <v>41</v>
+      </c>
+      <c r="B19" t="s">
+        <v>42</v>
+      </c>
+      <c r="C19" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3">
+      <c r="A20" t="s">
+        <v>43</v>
+      </c>
+      <c r="B20" t="s">
+        <v>44</v>
+      </c>
+      <c r="C20" t="s">
+        <v>34</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:C15" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:C20" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -953,28 +1041,28 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="B1" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="C1" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="D1" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="E1" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="F1" t="s">
         <v>0</v>
       </c>
       <c r="G1" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="H1" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -982,22 +1070,22 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="C2" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="D2" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="E2" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="F2" t="s">
         <v>3</v>
       </c>
       <c r="G2" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="H2" t="s">
         <v>3</v>
@@ -1010,33 +1098,33 @@
     </row>
     <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="C4" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="D4" t="s">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="E4" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="F4" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="G4" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="H4" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" t="s">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="B5" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="C5" t="b">
         <v>1</v>
@@ -1054,15 +1142,15 @@
         <v>4</v>
       </c>
       <c r="H5" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="B6" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="C6" t="b">
         <v>1</v>
@@ -1077,15 +1165,15 @@
         <v>5</v>
       </c>
       <c r="H6" t="s">
-        <v>57</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="B7" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="C7" t="b">
         <v>1</v>
@@ -1100,15 +1188,15 @@
         <v>5</v>
       </c>
       <c r="H7" t="s">
-        <v>59</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="B8" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="C8" t="b">
         <v>1</v>
@@ -1123,15 +1211,15 @@
         <v>5</v>
       </c>
       <c r="H8" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
     </row>
     <row r="9" spans="1:8">
       <c r="A9" t="s">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="B9" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="C9" t="b">
         <v>1</v>
@@ -1146,7 +1234,7 @@
         <v>5</v>
       </c>
       <c r="H9" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -1160,128 +1248,185 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:M13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
+  <cols>
+    <col min="7" max="7" width="19.85546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="B1" t="s">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="C1" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="D1" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="E1" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="F1" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="G1" t="s">
-        <v>0</v>
+        <v>78</v>
       </c>
       <c r="H1" t="s">
-        <v>40</v>
+        <v>79</v>
       </c>
       <c r="I1" t="s">
-        <v>41</v>
+        <v>80</v>
       </c>
       <c r="J1" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
       <c r="K1" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11">
+        <v>51</v>
+      </c>
+      <c r="L1" t="s">
+        <v>81</v>
+      </c>
+      <c r="M1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
       <c r="A2" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="D2" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="E2" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="F2" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="G2" t="s">
         <v>3</v>
       </c>
       <c r="H2" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="I2" t="s">
         <v>3</v>
       </c>
       <c r="J2" t="s">
-        <v>3</v>
+        <v>55</v>
       </c>
       <c r="K2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:11">
+      <c r="L2" t="s">
+        <v>3</v>
+      </c>
+      <c r="M2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
       <c r="A3" t="s">
         <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11">
+        <v>84</v>
+      </c>
+      <c r="C3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D3" t="s">
+        <v>85</v>
+      </c>
+      <c r="E3" t="s">
+        <v>85</v>
+      </c>
+      <c r="F3" t="s">
+        <v>85</v>
+      </c>
+      <c r="G3" t="s">
+        <v>85</v>
+      </c>
+      <c r="H3" t="s">
+        <v>85</v>
+      </c>
+      <c r="I3" t="s">
+        <v>85</v>
+      </c>
+      <c r="J3" t="s">
+        <v>85</v>
+      </c>
+      <c r="K3" t="s">
+        <v>85</v>
+      </c>
+      <c r="L3" t="s">
+        <v>85</v>
+      </c>
+      <c r="M3" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" t="s">
+        <v>85</v>
+      </c>
       <c r="B4" t="s">
-        <v>72</v>
+        <v>86</v>
       </c>
       <c r="C4" t="s">
-        <v>73</v>
+        <v>87</v>
       </c>
       <c r="D4" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="E4" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="F4" t="s">
-        <v>75</v>
+        <v>89</v>
       </c>
       <c r="G4" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="H4" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="I4" t="s">
-        <v>52</v>
+        <v>85</v>
       </c>
       <c r="J4" t="s">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="K4" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11">
+        <v>62</v>
+      </c>
+      <c r="L4" t="s">
+        <v>91</v>
+      </c>
+      <c r="M4" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
       <c r="A5">
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="C5" t="s">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="D5" t="b">
         <v>1</v>
@@ -1292,28 +1437,31 @@
       <c r="F5">
         <v>1</v>
       </c>
-      <c r="G5" t="s">
+      <c r="I5" t="s">
         <v>10</v>
       </c>
-      <c r="H5">
+      <c r="J5">
         <v>10</v>
       </c>
-      <c r="I5" t="s">
-        <v>82</v>
-      </c>
       <c r="K5" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11">
+        <v>96</v>
+      </c>
+      <c r="L5" t="s">
+        <v>85</v>
+      </c>
+      <c r="M5" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
       <c r="A6">
         <v>2</v>
       </c>
       <c r="B6" t="s">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="C6" t="s">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="D6" t="b">
         <v>1</v>
@@ -1324,25 +1472,31 @@
       <c r="F6">
         <v>1</v>
       </c>
-      <c r="G6" t="s">
+      <c r="I6" t="s">
         <v>10</v>
       </c>
-      <c r="H6">
+      <c r="J6">
         <v>40</v>
       </c>
-      <c r="I6" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11">
+      <c r="K6" t="s">
+        <v>98</v>
+      </c>
+      <c r="L6" t="s">
+        <v>85</v>
+      </c>
+      <c r="M6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
       <c r="A7">
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="C7" t="s">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="D7" t="b">
         <v>1</v>
@@ -1353,25 +1507,31 @@
       <c r="F7">
         <v>1</v>
       </c>
-      <c r="G7" t="s">
+      <c r="I7" t="s">
         <v>10</v>
       </c>
-      <c r="H7">
+      <c r="J7">
         <v>200</v>
       </c>
-      <c r="I7" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11">
+      <c r="K7" t="s">
+        <v>99</v>
+      </c>
+      <c r="L7" t="s">
+        <v>85</v>
+      </c>
+      <c r="M7" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
       <c r="A8">
         <v>4</v>
       </c>
       <c r="B8" t="s">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="C8" t="s">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="D8" t="b">
         <v>1</v>
@@ -1382,25 +1542,31 @@
       <c r="F8">
         <v>1</v>
       </c>
-      <c r="G8" t="s">
+      <c r="I8" t="s">
         <v>10</v>
       </c>
-      <c r="H8">
+      <c r="J8">
         <v>1000</v>
       </c>
-      <c r="I8" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11">
+      <c r="K8" t="s">
+        <v>100</v>
+      </c>
+      <c r="L8" t="s">
+        <v>85</v>
+      </c>
+      <c r="M8" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
       <c r="A9">
         <v>5</v>
       </c>
       <c r="B9" t="s">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="C9" t="s">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="D9" t="b">
         <v>1</v>
@@ -1411,25 +1577,31 @@
       <c r="F9">
         <v>1</v>
       </c>
-      <c r="G9" t="s">
+      <c r="I9" t="s">
         <v>10</v>
       </c>
-      <c r="H9">
+      <c r="J9">
         <v>5000</v>
       </c>
-      <c r="I9" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11">
+      <c r="K9" t="s">
+        <v>101</v>
+      </c>
+      <c r="L9" t="s">
+        <v>85</v>
+      </c>
+      <c r="M9" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
       <c r="A10">
         <v>6</v>
       </c>
       <c r="B10" t="s">
-        <v>88</v>
+        <v>102</v>
       </c>
       <c r="C10" t="s">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="D10" t="b">
         <v>1</v>
@@ -1441,24 +1613,36 @@
         <v>2</v>
       </c>
       <c r="G10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H10" t="s">
+        <v>95</v>
+      </c>
+      <c r="I10" t="s">
         <v>13</v>
       </c>
-      <c r="H10">
+      <c r="J10">
         <v>100</v>
       </c>
-      <c r="I10" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11">
+      <c r="K10" t="s">
+        <v>101</v>
+      </c>
+      <c r="L10" t="s">
+        <v>85</v>
+      </c>
+      <c r="M10" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13">
       <c r="A11">
         <v>7</v>
       </c>
       <c r="B11" t="s">
-        <v>89</v>
+        <v>103</v>
       </c>
       <c r="C11" t="s">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="D11" t="b">
         <v>1</v>
@@ -1470,24 +1654,36 @@
         <v>3</v>
       </c>
       <c r="G11" t="s">
+        <v>13</v>
+      </c>
+      <c r="H11" t="s">
+        <v>95</v>
+      </c>
+      <c r="I11" t="s">
         <v>15</v>
       </c>
-      <c r="H11">
+      <c r="J11">
         <v>100</v>
       </c>
-      <c r="I11" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11">
+      <c r="K11" t="s">
+        <v>101</v>
+      </c>
+      <c r="L11" t="s">
+        <v>85</v>
+      </c>
+      <c r="M11" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13">
       <c r="A12">
         <v>8</v>
       </c>
       <c r="B12" t="s">
-        <v>90</v>
+        <v>104</v>
       </c>
       <c r="C12" t="s">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="D12" t="b">
         <v>1</v>
@@ -1499,24 +1695,36 @@
         <v>4</v>
       </c>
       <c r="G12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H12" t="s">
+        <v>95</v>
+      </c>
+      <c r="I12" t="s">
         <v>17</v>
       </c>
-      <c r="H12">
+      <c r="J12">
         <v>100</v>
       </c>
-      <c r="I12" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11">
+      <c r="K12" t="s">
+        <v>101</v>
+      </c>
+      <c r="L12" t="s">
+        <v>85</v>
+      </c>
+      <c r="M12" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13">
       <c r="A13">
         <v>9</v>
       </c>
       <c r="B13" t="s">
-        <v>91</v>
+        <v>105</v>
       </c>
       <c r="C13" t="s">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="D13" t="b">
         <v>1</v>
@@ -1528,133 +1736,127 @@
         <v>5</v>
       </c>
       <c r="G13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H13" t="s">
+        <v>95</v>
+      </c>
+      <c r="I13" t="s">
         <v>19</v>
       </c>
-      <c r="H13">
+      <c r="J13">
         <v>100</v>
       </c>
-      <c r="I13" t="s">
-        <v>87</v>
+      <c r="K13" t="s">
+        <v>101</v>
+      </c>
+      <c r="L13" t="s">
+        <v>85</v>
+      </c>
+      <c r="M13" t="s">
+        <v>85</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:K13" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:M4 A13:F13 A5:F9 I5:M9 A10:F10 H10:M10 A11:F11 H11:M11 A12:F12 H12:M12 H13:M13" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
-  <cols>
-    <col min="1" max="1" width="20.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.140625" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="19" customWidth="1"/>
-    <col min="6" max="7" width="23" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="30.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="30.5703125" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:8">
       <c r="A1" t="s">
-        <v>92</v>
+        <v>106</v>
       </c>
       <c r="B1" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
       </c>
       <c r="D1" t="s">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="E1" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="F1" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
       <c r="G1" t="s">
-        <v>98</v>
+        <v>110</v>
       </c>
       <c r="H1" t="s">
-        <v>93</v>
-      </c>
-      <c r="I1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2" t="s">
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="C2" t="s">
         <v>3</v>
       </c>
       <c r="D2" t="s">
+        <v>112</v>
+      </c>
+      <c r="E2" t="s">
+        <v>113</v>
+      </c>
+      <c r="F2" t="s">
+        <v>113</v>
+      </c>
+      <c r="G2" t="s">
         <v>3</v>
-      </c>
-      <c r="E2" t="s">
-        <v>99</v>
-      </c>
-      <c r="F2" t="s">
-        <v>100</v>
-      </c>
-      <c r="G2" t="s">
-        <v>100</v>
       </c>
       <c r="H2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9">
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>101</v>
+        <v>114</v>
       </c>
       <c r="B4" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="C4" t="s">
-        <v>102</v>
+        <v>115</v>
       </c>
       <c r="D4" t="s">
-        <v>105</v>
+        <v>116</v>
       </c>
       <c r="E4" t="s">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="F4" t="s">
-        <v>107</v>
+        <v>118</v>
       </c>
       <c r="G4" t="s">
-        <v>108</v>
+        <v>119</v>
       </c>
       <c r="H4" t="s">
-        <v>103</v>
-      </c>
-      <c r="I4" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
       <c r="A5" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
       <c r="B5" t="b">
         <v>1</v>
@@ -1663,26 +1865,23 @@
         <v>32</v>
       </c>
       <c r="D5" t="s">
-        <v>111</v>
+        <v>122</v>
       </c>
       <c r="E5" t="s">
-        <v>112</v>
+        <v>123</v>
       </c>
       <c r="F5" t="s">
-        <v>113</v>
-      </c>
-      <c r="G5" t="s">
-        <v>114</v>
-      </c>
-      <c r="I5" t="s">
-        <v>110</v>
+        <v>124</v>
+      </c>
+      <c r="H5" t="s">
+        <v>125</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:C5 D1:G5" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:H5" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1691,39 +1890,36 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
-  <cols>
-    <col min="2" max="2" width="35.85546875" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="B1" t="s">
-        <v>92</v>
+        <v>106</v>
       </c>
       <c r="C1" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="D1" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="E1" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>117</v>
+        <v>128</v>
       </c>
       <c r="D2" t="s">
-        <v>117</v>
+        <v>128</v>
       </c>
       <c r="E2" t="s">
         <v>3</v>
@@ -1734,24 +1930,24 @@
         <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="B4" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="C4" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="D4" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="E4" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -1759,7 +1955,7 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
       <c r="C5">
         <v>1</v>
@@ -1768,7 +1964,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="s">
-        <v>86</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -1776,7 +1972,7 @@
         <v>2</v>
       </c>
       <c r="B6" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
       <c r="C6">
         <v>11</v>
@@ -1785,7 +1981,7 @@
         <v>100</v>
       </c>
       <c r="E6" t="s">
-        <v>87</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>